<commit_message>
save 14 08 2026
</commit_message>
<xml_diff>
--- a/3 четверть_2_Java Development Kit.xlsx
+++ b/3 четверть_2_Java Development Kit.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Machenike\Desktop\Homework_repo\GB_Developer_Workbook\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AlexServHW\Desktop\GB_Developer_Workbook\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75D70FD9-2A31-4F1F-92CE-9F83E8A4C3AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7788EBD0-6587-4B6E-889F-6E2205336309}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-10545" yWindow="-19635" windowWidth="23010" windowHeight="16845" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Название 1-3" sheetId="12" r:id="rId1"/>
@@ -19,6 +19,9 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -5295,33 +5298,6 @@
   </si>
   <si>
     <t>Лучше скопировать из конспекта к лекции</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="204"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Важно! Данимическая типизация в Java</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-&lt;Number&gt; может быть только new c Number
-&lt;? extends Number&gt; может быть new с Number или его наследниками
-&lt;? super Number&gt; может быть new с Number или его родителями</t>
-    </r>
   </si>
   <si>
     <r>
@@ -10048,25 +10024,44 @@
   <si>
     <t>Способ 3 : заставляем поток main ожидать другие потоки. Через оператор ввода пользователя. Бесполезен в больших программах</t>
   </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="204"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Важно! Динамическая типизация в Java</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+&lt;Number&gt; может быть только new c Number
+&lt;? extends Number&gt; может быть new с Number или его наследниками
+&lt;? super Number&gt; может быть new с Number или его родителями</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="33" x14ac:knownFonts="1">
+  <fonts count="32" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="204"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -10630,29 +10625,29 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="97">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="25" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -10664,13 +10659,13 @@
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="22" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -10679,61 +10674,61 @@
     <xf numFmtId="49" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="20" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="20" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="18" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="19" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="32" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="17" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -10742,19 +10737,10 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -10763,7 +10749,13 @@
     <xf numFmtId="49" fontId="13" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -10772,7 +10764,7 @@
     <xf numFmtId="49" fontId="11" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="26" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -10790,7 +10782,7 @@
     <xf numFmtId="49" fontId="9" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="25" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -10811,7 +10803,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="27" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="26" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -10841,7 +10833,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="25" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -10859,7 +10851,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="29" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="28" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
@@ -10892,7 +10884,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="25" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="18" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -10920,6 +10912,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -12224,48 +12219,48 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:U443"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="36" style="1" customWidth="1"/>
-    <col min="2" max="2" width="50.54296875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="71.1796875" style="2" customWidth="1"/>
-    <col min="4" max="4" width="56.453125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="6.26953125" style="8" customWidth="1"/>
-    <col min="6" max="6" width="43.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="55.08984375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="67.90625" style="1" customWidth="1"/>
-    <col min="9" max="9" width="64.36328125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="7.81640625" style="8" customWidth="1"/>
-    <col min="11" max="11" width="39.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="48.90625" style="1" customWidth="1"/>
-    <col min="13" max="13" width="72.6328125" style="1" customWidth="1"/>
-    <col min="14" max="14" width="43.90625" style="1" customWidth="1"/>
-    <col min="15" max="15" width="7.81640625" style="8" customWidth="1"/>
-    <col min="16" max="16" width="56.81640625" style="1" customWidth="1"/>
-    <col min="17" max="17" width="46.7265625" style="1" customWidth="1"/>
-    <col min="18" max="18" width="62.90625" style="1" customWidth="1"/>
-    <col min="19" max="19" width="49.1796875" style="1" customWidth="1"/>
-    <col min="20" max="20" width="8.7265625" style="9"/>
-    <col min="21" max="21" width="67.7265625" style="1" customWidth="1"/>
-    <col min="22" max="22" width="68.36328125" style="1" customWidth="1"/>
-    <col min="23" max="24" width="59.36328125" style="1" customWidth="1"/>
-    <col min="25" max="25" width="59.6328125" style="1" customWidth="1"/>
-    <col min="26" max="26" width="99.453125" style="1" customWidth="1"/>
-    <col min="27" max="27" width="41.26953125" style="1" customWidth="1"/>
-    <col min="28" max="16384" width="8.7265625" style="1"/>
+    <col min="2" max="2" width="50.5546875" style="1" customWidth="1"/>
+    <col min="3" max="3" width="71.21875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="56.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="6.21875" style="8" customWidth="1"/>
+    <col min="6" max="6" width="43.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="55.109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="67.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="64.33203125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="7.77734375" style="8" customWidth="1"/>
+    <col min="11" max="11" width="39.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="48.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="72.6640625" style="1" customWidth="1"/>
+    <col min="14" max="14" width="43.88671875" style="1" customWidth="1"/>
+    <col min="15" max="15" width="7.77734375" style="8" customWidth="1"/>
+    <col min="16" max="16" width="56.77734375" style="1" customWidth="1"/>
+    <col min="17" max="17" width="46.77734375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="62.88671875" style="1" customWidth="1"/>
+    <col min="19" max="19" width="49.21875" style="1" customWidth="1"/>
+    <col min="20" max="20" width="8.77734375" style="9"/>
+    <col min="21" max="21" width="67.77734375" style="1" customWidth="1"/>
+    <col min="22" max="22" width="68.33203125" style="1" customWidth="1"/>
+    <col min="23" max="24" width="59.33203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="59.6640625" style="1" customWidth="1"/>
+    <col min="26" max="26" width="99.44140625" style="1" customWidth="1"/>
+    <col min="27" max="27" width="41.21875" style="1" customWidth="1"/>
+    <col min="28" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" s="25" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="4"/>
@@ -12284,7 +12279,7 @@
       <c r="S6" s="3"/>
       <c r="U6" s="3"/>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>0</v>
       </c>
@@ -12292,7 +12287,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
         <v>1</v>
       </c>
@@ -12300,7 +12295,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -12308,7 +12303,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -12316,7 +12311,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
         <v>5</v>
       </c>
@@ -12324,7 +12319,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12" s="10" t="s">
         <v>9</v>
       </c>
@@ -12332,7 +12327,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>16</v>
       </c>
@@ -12340,7 +12335,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>14</v>
       </c>
@@ -12354,7 +12349,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A15" s="7" t="s">
         <v>19</v>
       </c>
@@ -12365,12 +12360,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" s="10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:21" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:21" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>26</v>
       </c>
@@ -12384,7 +12379,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="18" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>24</v>
       </c>
@@ -12392,7 +12387,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="19" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>23</v>
       </c>
@@ -12400,7 +12395,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A20" s="10" t="s">
         <v>27</v>
       </c>
@@ -12408,7 +12403,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:21" ht="203" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:21" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>30</v>
       </c>
@@ -12416,7 +12411,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:21" ht="261" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:21" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>31</v>
       </c>
@@ -12428,7 +12423,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>34</v>
       </c>
@@ -12436,7 +12431,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="24" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>33</v>
       </c>
@@ -12444,7 +12439,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="25" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>35</v>
       </c>
@@ -12452,13 +12447,13 @@
         <v>52</v>
       </c>
     </row>
-    <row r="26" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="10" t="s">
         <v>40</v>
       </c>
       <c r="C26" s="6"/>
     </row>
-    <row r="27" spans="1:21" ht="145" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:21" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>39</v>
       </c>
@@ -12472,7 +12467,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="4"/>
@@ -12491,7 +12486,7 @@
       <c r="S28" s="3"/>
       <c r="U28" s="3"/>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>43</v>
       </c>
@@ -12500,7 +12495,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="30" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="10" t="s">
         <v>45</v>
       </c>
@@ -12508,7 +12503,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="31" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>47</v>
       </c>
@@ -12516,7 +12511,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="32" spans="1:21" ht="58" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>46</v>
       </c>
@@ -12524,7 +12519,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="10" t="s">
         <v>48</v>
       </c>
@@ -12535,7 +12530,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="348" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:4" ht="345.6" x14ac:dyDescent="0.3">
       <c r="B34" s="1" t="s">
         <v>50</v>
       </c>
@@ -12543,7 +12538,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="35" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>79</v>
       </c>
@@ -12551,7 +12546,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="10" t="s">
         <v>60</v>
       </c>
@@ -12559,12 +12554,12 @@
         <v>58</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:4" ht="72" x14ac:dyDescent="0.3">
       <c r="C37" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="38" spans="1:4" ht="87" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>62</v>
       </c>
@@ -12575,7 +12570,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A39" s="12" t="s">
         <v>72</v>
       </c>
@@ -12586,7 +12581,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="174" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:4" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>63</v>
       </c>
@@ -12597,17 +12592,17 @@
         <v>76</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>66</v>
       </c>
@@ -12618,12 +12613,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="45" spans="1:4" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>68</v>
       </c>
@@ -12634,17 +12629,17 @@
         <v>83</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="10" t="s">
         <v>81</v>
       </c>
@@ -12655,12 +12650,12 @@
         <v>78</v>
       </c>
     </row>
-    <row r="49" spans="1:21" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:21" ht="172.8" x14ac:dyDescent="0.3">
       <c r="C49" s="6" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A50" s="10" t="s">
         <v>89</v>
       </c>
@@ -12668,12 +12663,12 @@
         <v>88</v>
       </c>
     </row>
-    <row r="51" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C51" s="6" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="52" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>91</v>
       </c>
@@ -12681,7 +12676,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="53" spans="1:21" ht="190.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:21" ht="190.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="15" t="s">
         <v>131</v>
       </c>
@@ -12692,7 +12687,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="54" spans="1:21" ht="70.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:21" ht="70.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B54" s="15" t="s">
         <v>132</v>
       </c>
@@ -12703,7 +12698,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="55" spans="1:21" ht="144.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:21" ht="144.44999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B55" s="15" t="s">
         <v>133</v>
       </c>
@@ -12711,7 +12706,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>97</v>
       </c>
@@ -12720,7 +12715,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="57" spans="1:21" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>98</v>
       </c>
@@ -12731,7 +12726,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="58" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A58" s="10" t="s">
         <v>143</v>
       </c>
@@ -12740,7 +12735,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="59" spans="1:21" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:21" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A59" s="17" t="s">
         <v>144</v>
       </c>
@@ -12754,7 +12749,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="60" spans="1:21" ht="145" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:21" ht="144" x14ac:dyDescent="0.3">
       <c r="B60" s="15" t="s">
         <v>136</v>
       </c>
@@ -12762,12 +12757,12 @@
         <v>110</v>
       </c>
     </row>
-    <row r="61" spans="1:21" ht="58" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B61" s="15" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="62" spans="1:21" ht="145" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:21" ht="144" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>140</v>
       </c>
@@ -12778,12 +12773,12 @@
         <v>141</v>
       </c>
     </row>
-    <row r="63" spans="1:21" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:21" ht="187.2" x14ac:dyDescent="0.3">
       <c r="B63" s="19" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="64" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="4"/>
@@ -12802,7 +12797,7 @@
       <c r="S64" s="3"/>
       <c r="U64" s="3"/>
     </row>
-    <row r="65" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>101</v>
       </c>
@@ -12811,7 +12806,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="66" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A66" s="10" t="s">
         <v>102</v>
       </c>
@@ -12819,7 +12814,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="67" spans="1:21" ht="174" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:21" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>124</v>
       </c>
@@ -12830,7 +12825,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="68" spans="1:21" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:21" ht="129.6" x14ac:dyDescent="0.3">
       <c r="B68" s="14" t="s">
         <v>127</v>
       </c>
@@ -12838,7 +12833,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="69" spans="1:21" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:21" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
         <v>115</v>
       </c>
@@ -12849,7 +12844,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="70" spans="1:21" ht="81.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:21" ht="81.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>117</v>
       </c>
@@ -12860,7 +12855,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="71" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>116</v>
       </c>
@@ -12869,7 +12864,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="72" spans="1:21" ht="116" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:21" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>106</v>
       </c>
@@ -12883,7 +12878,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="73" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>119</v>
       </c>
@@ -12892,7 +12887,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="74" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A74" s="10" t="s">
         <v>122</v>
       </c>
@@ -12901,7 +12896,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="75" spans="1:21" ht="261" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:21" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A75" s="17" t="s">
         <v>123</v>
       </c>
@@ -12915,12 +12910,12 @@
         <v>108</v>
       </c>
     </row>
-    <row r="76" spans="1:21" ht="159.5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:21" ht="158.4" x14ac:dyDescent="0.3">
       <c r="C76" s="17" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="78" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
       <c r="C78" s="4"/>
@@ -12939,7 +12934,7 @@
       <c r="S78" s="3"/>
       <c r="U78" s="3"/>
     </row>
-    <row r="79" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>112</v>
       </c>
@@ -12948,7 +12943,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="80" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B80" s="1" t="s">
         <v>151</v>
       </c>
@@ -12956,7 +12951,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="83" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="4"/>
@@ -12975,7 +12970,7 @@
       <c r="S83" s="3"/>
       <c r="U83" s="3"/>
     </row>
-    <row r="84" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>147</v>
       </c>
@@ -12986,12 +12981,12 @@
         <v>148</v>
       </c>
     </row>
-    <row r="85" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C85" s="23" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="86" spans="1:21" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:21" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
         <v>159</v>
       </c>
@@ -13005,7 +13000,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="87" spans="1:21" ht="58" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>164</v>
       </c>
@@ -13016,7 +13011,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="88" spans="1:21" ht="377" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:21" ht="374.4" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>165</v>
       </c>
@@ -13030,17 +13025,17 @@
         <v>163</v>
       </c>
     </row>
-    <row r="89" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A89" s="10" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="90" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="91" spans="1:21" ht="275.5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:21" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>170</v>
       </c>
@@ -13054,7 +13049,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="92" spans="1:21" ht="188.5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:21" ht="187.2" x14ac:dyDescent="0.3">
       <c r="B92" s="1" t="s">
         <v>174</v>
       </c>
@@ -13062,7 +13057,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="93" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C93" s="28" t="s">
         <v>176</v>
       </c>
@@ -13070,7 +13065,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="94" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C94" s="28" t="s">
         <v>178</v>
       </c>
@@ -13078,7 +13073,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="95" spans="1:21" ht="145" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:21" ht="144" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>181</v>
       </c>
@@ -13089,7 +13084,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="96" spans="1:21" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A96" s="27" t="s">
         <v>184</v>
       </c>
@@ -13103,7 +13098,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="97" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
       <c r="C97" s="4"/>
@@ -13122,7 +13117,7 @@
       <c r="S97" s="3"/>
       <c r="U97" s="3"/>
     </row>
-    <row r="98" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>189</v>
       </c>
@@ -13130,7 +13125,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="99" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A99" s="10" t="s">
         <v>187</v>
       </c>
@@ -13138,7 +13133,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="100" spans="1:21" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
       <c r="B100" s="32" t="s">
         <v>206</v>
       </c>
@@ -13149,7 +13144,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="101" spans="1:21" ht="174" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:21" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A101" s="29" t="s">
         <v>191</v>
       </c>
@@ -13160,12 +13155,12 @@
         <v>192</v>
       </c>
     </row>
-    <row r="102" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C102" s="27" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="103" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A103" s="10" t="s">
         <v>195</v>
       </c>
@@ -13176,7 +13171,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="104" spans="1:21" ht="232" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:21" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>198</v>
       </c>
@@ -13187,7 +13182,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="105" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A105" s="3"/>
       <c r="B105" s="3"/>
       <c r="C105" s="4"/>
@@ -13206,7 +13201,7 @@
       <c r="S105" s="3"/>
       <c r="U105" s="3"/>
     </row>
-    <row r="106" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>201</v>
       </c>
@@ -13217,13 +13212,13 @@
         <v>203</v>
       </c>
     </row>
-    <row r="107" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A107" s="10" t="s">
         <v>202</v>
       </c>
       <c r="C107" s="27"/>
     </row>
-    <row r="108" spans="1:21" ht="145" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:21" ht="144" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>181</v>
       </c>
@@ -13231,7 +13226,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="109" spans="1:21" ht="145" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:21" ht="144" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>181</v>
       </c>
@@ -13239,7 +13234,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="113" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A113" s="3"/>
       <c r="B113" s="3"/>
       <c r="C113" s="4"/>
@@ -13258,7 +13253,7 @@
       <c r="S113" s="3"/>
       <c r="U113" s="3"/>
     </row>
-    <row r="114" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>208</v>
       </c>
@@ -13266,7 +13261,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="115" spans="1:21" ht="58" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B115" s="34" t="s">
         <v>213</v>
       </c>
@@ -13277,12 +13272,12 @@
         <v>211</v>
       </c>
     </row>
-    <row r="116" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C116" s="34" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="117" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A117" s="7" t="s">
         <v>214</v>
       </c>
@@ -13290,17 +13285,17 @@
         <v>217</v>
       </c>
     </row>
-    <row r="118" spans="1:21" ht="58" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="C118" s="34" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="119" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C119" s="34" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="120" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A120" s="10" t="s">
         <v>218</v>
       </c>
@@ -13308,12 +13303,12 @@
         <v>220</v>
       </c>
     </row>
-    <row r="121" spans="1:21" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:21" ht="129.6" x14ac:dyDescent="0.3">
       <c r="C121" s="34" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="122" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A122" s="35" t="s">
         <v>221</v>
       </c>
@@ -13323,20 +13318,20 @@
         <v>222</v>
       </c>
     </row>
-    <row r="123" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A123" s="10" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="124" spans="1:21" ht="87" x14ac:dyDescent="0.35">
-      <c r="B124" s="45" t="s">
-        <v>340</v>
+    <row r="124" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="B124" s="44" t="s">
+        <v>339</v>
       </c>
       <c r="C124" s="34" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="125" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A125" s="3"/>
       <c r="B125" s="3"/>
       <c r="C125" s="4"/>
@@ -13355,7 +13350,7 @@
       <c r="S125" s="3"/>
       <c r="U125" s="3"/>
     </row>
-    <row r="126" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
         <v>246</v>
       </c>
@@ -13363,7 +13358,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="127" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A127" s="10" t="s">
         <v>225</v>
       </c>
@@ -13371,7 +13366,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="128" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="B128" s="34" t="s">
         <v>228</v>
       </c>
@@ -13379,17 +13374,17 @@
         <v>227</v>
       </c>
     </row>
-    <row r="129" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A129" s="10" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="130" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="C130" s="34" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="131" spans="1:21" ht="58" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A131" s="10" t="s">
         <v>231</v>
       </c>
@@ -13397,12 +13392,12 @@
         <v>232</v>
       </c>
     </row>
-    <row r="132" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C132" s="33" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="133" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="A133" s="34" t="s">
         <v>234</v>
       </c>
@@ -13416,7 +13411,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="134" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A134" s="10" t="s">
         <v>237</v>
       </c>
@@ -13424,7 +13419,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="135" spans="1:21" ht="58" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B135" s="34" t="s">
         <v>240</v>
       </c>
@@ -13432,7 +13427,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="136" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A136" s="10" t="s">
         <v>241</v>
       </c>
@@ -13440,12 +13435,12 @@
         <v>94</v>
       </c>
     </row>
-    <row r="137" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="B137" s="34" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="138" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A138" s="3"/>
       <c r="B138" s="3"/>
       <c r="C138" s="4"/>
@@ -13464,7 +13459,7 @@
       <c r="S138" s="3"/>
       <c r="U138" s="3"/>
     </row>
-    <row r="139" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
         <v>247</v>
       </c>
@@ -13475,53 +13470,53 @@
         <v>244</v>
       </c>
     </row>
-    <row r="140" spans="1:21" ht="145" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:21" ht="144" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="B140" s="44" t="s">
         <v>341</v>
       </c>
-      <c r="B140" s="45" t="s">
+      <c r="C140" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="C140" s="1" t="s">
+    </row>
+    <row r="141" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B141" s="44"/>
+      <c r="C141" s="10" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="141" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="B141" s="45"/>
-      <c r="C141" s="10" t="s">
+      <c r="D141" s="10" t="s">
         <v>344</v>
       </c>
-      <c r="D141" s="10" t="s">
+    </row>
+    <row r="142" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B142" s="44"/>
+      <c r="C142" s="1" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="142" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="B142" s="45"/>
-      <c r="C142" s="1" t="s">
+      <c r="D142" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="D142" s="1" t="s">
+    </row>
+    <row r="143" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B143" s="44"/>
+      <c r="C143" s="1" t="s">
         <v>347</v>
       </c>
-    </row>
-    <row r="143" spans="1:21" ht="58" x14ac:dyDescent="0.35">
-      <c r="B143" s="45"/>
-      <c r="C143" s="1" t="s">
+      <c r="D143" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="D143" s="1" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="144" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="B144" s="45"/>
-      <c r="C144" s="45"/>
-    </row>
-    <row r="145" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="B145" s="45"/>
-      <c r="C145" s="45"/>
-    </row>
-    <row r="146" spans="1:21" x14ac:dyDescent="0.35">
+    </row>
+    <row r="144" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B144" s="44"/>
+      <c r="C144" s="44"/>
+    </row>
+    <row r="145" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="B145" s="44"/>
+      <c r="C145" s="44"/>
+    </row>
+    <row r="146" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A146" s="3"/>
       <c r="B146" s="3"/>
       <c r="C146" s="4"/>
@@ -13540,7 +13535,7 @@
       <c r="S146" s="3"/>
       <c r="U146" s="3"/>
     </row>
-    <row r="147" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A147" s="1" t="s">
         <v>249</v>
       </c>
@@ -13551,12 +13546,12 @@
         <v>251</v>
       </c>
     </row>
-    <row r="148" spans="1:21" ht="87" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="C148" s="34" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="149" spans="1:21" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:21" ht="129.6" x14ac:dyDescent="0.3">
       <c r="B149" s="34" t="s">
         <v>254</v>
       </c>
@@ -13564,7 +13559,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="150" spans="1:21" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
       <c r="B150" s="34" t="s">
         <v>256</v>
       </c>
@@ -13572,7 +13567,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="151" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A151" s="10" t="s">
         <v>268</v>
       </c>
@@ -13580,7 +13575,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="152" spans="1:21" ht="87" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B152" s="39" t="s">
         <v>270</v>
       </c>
@@ -13591,7 +13586,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="153" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="B153" s="39" t="s">
         <v>272</v>
       </c>
@@ -13599,19 +13594,19 @@
         <v>271</v>
       </c>
     </row>
-    <row r="154" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B154" s="34"/>
       <c r="C154" s="34"/>
     </row>
-    <row r="155" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B155" s="34"/>
       <c r="C155" s="34"/>
     </row>
-    <row r="156" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B156" s="34"/>
       <c r="C156" s="34"/>
     </row>
-    <row r="157" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A157" s="3"/>
       <c r="B157" s="3"/>
       <c r="C157" s="4"/>
@@ -13630,7 +13625,7 @@
       <c r="S157" s="3"/>
       <c r="U157" s="3"/>
     </row>
-    <row r="158" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A158" s="1" t="s">
         <v>257</v>
       </c>
@@ -13641,7 +13636,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="159" spans="1:21" ht="174" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:21" ht="172.8" x14ac:dyDescent="0.3">
       <c r="B159" s="34" t="s">
         <v>261</v>
       </c>
@@ -13649,12 +13644,12 @@
         <v>259</v>
       </c>
     </row>
-    <row r="160" spans="1:21" ht="217.5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:21" ht="187.2" x14ac:dyDescent="0.3">
       <c r="C160" s="34" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="161" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A161" s="10" t="s">
         <v>263</v>
       </c>
@@ -13665,12 +13660,12 @@
         <v>264</v>
       </c>
     </row>
-    <row r="162" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C162" s="34" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="164" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A164" s="3"/>
       <c r="B164" s="3"/>
       <c r="C164" s="4"/>
@@ -13689,7 +13684,7 @@
       <c r="S164" s="3"/>
       <c r="U164" s="3"/>
     </row>
-    <row r="165" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
         <v>273</v>
       </c>
@@ -13700,12 +13695,12 @@
         <v>275</v>
       </c>
     </row>
-    <row r="166" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C166" s="39" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="167" spans="1:21" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
       <c r="B167" s="39" t="s">
         <v>278</v>
       </c>
@@ -13713,7 +13708,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="168" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A168" s="10" t="s">
         <v>279</v>
       </c>
@@ -13721,12 +13716,12 @@
         <v>283</v>
       </c>
     </row>
-    <row r="169" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C169" s="1" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="170" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B170" s="41" t="s">
         <v>284</v>
       </c>
@@ -13734,12 +13729,12 @@
         <v>281</v>
       </c>
     </row>
-    <row r="171" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C171" s="1" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="172" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A172" s="3"/>
       <c r="B172" s="3"/>
       <c r="C172" s="4"/>
@@ -13758,7 +13753,7 @@
       <c r="S172" s="3"/>
       <c r="U172" s="3"/>
     </row>
-    <row r="173" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A173" s="1" t="s">
         <v>273</v>
       </c>
@@ -13769,12 +13764,12 @@
         <v>286</v>
       </c>
     </row>
-    <row r="174" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C174" s="39" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="175" spans="1:21" ht="333.5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:21" ht="331.2" x14ac:dyDescent="0.3">
       <c r="B175" s="39" t="s">
         <v>289</v>
       </c>
@@ -13782,7 +13777,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="176" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A176" s="3"/>
       <c r="B176" s="3"/>
       <c r="C176" s="4"/>
@@ -13801,7 +13796,7 @@
       <c r="S176" s="3"/>
       <c r="U176" s="3"/>
     </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A177" s="1" t="s">
         <v>291</v>
       </c>
@@ -13812,12 +13807,12 @@
         <v>292</v>
       </c>
     </row>
-    <row r="178" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C178" s="39" t="s">
         <v>293</v>
       </c>
     </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A179" s="10" t="s">
         <v>294</v>
       </c>
@@ -13828,7 +13823,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="180" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B180" s="39" t="s">
         <v>298</v>
       </c>
@@ -13836,17 +13831,17 @@
         <v>296</v>
       </c>
     </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C181" s="39" t="s">
         <v>297</v>
       </c>
     </row>
-    <row r="182" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C182" s="39" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="183" spans="1:4" ht="101.5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:4" ht="100.8" x14ac:dyDescent="0.3">
       <c r="B183" s="42" t="s">
         <v>303</v>
       </c>
@@ -13854,7 +13849,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="184" spans="1:4" ht="87" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:4" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A184" s="1" t="s">
         <v>324</v>
       </c>
@@ -13864,19 +13859,19 @@
       <c r="C184" s="42" t="s">
         <v>323</v>
       </c>
-      <c r="D184" s="44" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D184" s="96" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="185" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B185" s="42"/>
       <c r="C185" s="39"/>
     </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:4" x14ac:dyDescent="0.3">
       <c r="B186" s="42"/>
       <c r="C186" s="39"/>
     </row>
-    <row r="187" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A187" s="10" t="s">
         <v>304</v>
       </c>
@@ -13884,7 +13879,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="188" spans="1:4" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A188" s="7" t="s">
         <v>306</v>
       </c>
@@ -13892,7 +13887,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="189" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A189" s="7" t="s">
         <v>307</v>
       </c>
@@ -13900,7 +13895,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A190" s="7" t="s">
         <v>310</v>
       </c>
@@ -13908,27 +13903,27 @@
         <v>314</v>
       </c>
     </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:4" x14ac:dyDescent="0.3">
       <c r="C191" s="42" t="s">
         <v>315</v>
       </c>
     </row>
-    <row r="192" spans="1:4" ht="29" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C192" s="42" t="s">
         <v>311</v>
       </c>
     </row>
-    <row r="193" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C193" s="42" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="194" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:21" x14ac:dyDescent="0.3">
       <c r="C194" s="42" t="s">
         <v>313</v>
       </c>
     </row>
-    <row r="195" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A195" s="1" t="s">
         <v>316</v>
       </c>
@@ -13939,7 +13934,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="196" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A196" s="3"/>
       <c r="B196" s="3"/>
       <c r="C196" s="4"/>
@@ -13958,7 +13953,7 @@
       <c r="S196" s="3"/>
       <c r="U196" s="3"/>
     </row>
-    <row r="197" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A197" s="1" t="s">
         <v>321</v>
       </c>
@@ -13969,12 +13964,12 @@
         <v>319</v>
       </c>
     </row>
-    <row r="198" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
       <c r="C198" s="42" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="199" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A199" s="1" t="s">
         <v>326</v>
       </c>
@@ -13982,7 +13977,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="200" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A200" s="1" t="s">
         <v>327</v>
       </c>
@@ -13993,7 +13988,7 @@
         <v>328</v>
       </c>
     </row>
-    <row r="201" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A201" s="10" t="s">
         <v>331</v>
       </c>
@@ -14001,7 +13996,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="202" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:21" ht="72" x14ac:dyDescent="0.3">
       <c r="B202" s="42" t="s">
         <v>333</v>
       </c>
@@ -14009,7 +14004,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="203" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A203" s="3"/>
       <c r="B203" s="3"/>
       <c r="C203" s="4"/>
@@ -14028,7 +14023,7 @@
       <c r="S203" s="3"/>
       <c r="U203" s="3"/>
     </row>
-    <row r="204" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A204" s="1" t="s">
         <v>335</v>
       </c>
@@ -14039,12 +14034,12 @@
         <v>337</v>
       </c>
     </row>
-    <row r="205" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:21" x14ac:dyDescent="0.3">
       <c r="B205" s="41" t="s">
         <v>338</v>
       </c>
     </row>
-    <row r="208" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A208" s="3"/>
       <c r="B208" s="3"/>
       <c r="C208" s="4"/>
@@ -14063,49 +14058,49 @@
       <c r="S208" s="3"/>
       <c r="U208" s="3"/>
     </row>
-    <row r="209" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A209" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="C209" s="49" t="s">
-        <v>366</v>
+        <v>349</v>
+      </c>
+      <c r="C209" s="48" t="s">
+        <v>365</v>
       </c>
       <c r="D209" s="1" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="210" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A210" s="47" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="210" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A210" s="46" t="s">
+        <v>360</v>
+      </c>
+      <c r="B210" s="36"/>
+      <c r="C210" s="47" t="s">
+        <v>358</v>
+      </c>
+      <c r="D210" s="38" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="211" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A211" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="D211" s="1" t="s">
         <v>361</v>
       </c>
-      <c r="B210" s="36"/>
-      <c r="C210" s="48" t="s">
-        <v>359</v>
-      </c>
-      <c r="D210" s="38" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="211" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A211" s="10" t="s">
+    </row>
+    <row r="212" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A212" s="1" t="s">
         <v>363</v>
       </c>
-      <c r="D211" s="1" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="212" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A212" s="1" t="s">
+      <c r="C212" s="44"/>
+    </row>
+    <row r="213" spans="1:21" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A213" s="1" t="s">
         <v>364</v>
       </c>
-      <c r="C212" s="45"/>
-    </row>
-    <row r="213" spans="1:21" ht="130.5" x14ac:dyDescent="0.35">
-      <c r="A213" s="1" t="s">
-        <v>365</v>
-      </c>
-    </row>
-    <row r="215" spans="1:21" x14ac:dyDescent="0.35">
+    </row>
+    <row r="215" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A215" s="3"/>
       <c r="B215" s="3"/>
       <c r="C215" s="4"/>
@@ -14124,82 +14119,82 @@
       <c r="S215" s="3"/>
       <c r="U215" s="3"/>
     </row>
-    <row r="216" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A216" s="1" t="s">
-        <v>356</v>
-      </c>
-      <c r="C216" s="46" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="217" spans="1:21" ht="275.5" x14ac:dyDescent="0.35">
+        <v>355</v>
+      </c>
+      <c r="C216" s="45" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="217" spans="1:21" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A217" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="C217" s="49" t="s">
         <v>368</v>
       </c>
-      <c r="C217" s="50" t="s">
+    </row>
+    <row r="218" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A218" s="10" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="218" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A218" s="10" t="s">
+    <row r="219" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="B219" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="C219" s="49" t="s">
         <v>370</v>
       </c>
-    </row>
-    <row r="219" spans="1:21" ht="87" x14ac:dyDescent="0.35">
-      <c r="B219" s="1" t="s">
+      <c r="D219" s="1" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="220" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A220" s="10" t="s">
         <v>373</v>
       </c>
-      <c r="C219" s="50" t="s">
-        <v>371</v>
-      </c>
-      <c r="D219" s="1" t="s">
-        <v>372</v>
-      </c>
-    </row>
-    <row r="220" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A220" s="10" t="s">
+      <c r="D220" s="1" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="221" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B221" s="1" t="s">
+        <v>379</v>
+      </c>
+      <c r="C221" s="49" t="s">
+        <v>376</v>
+      </c>
+      <c r="D221" s="1" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="222" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A222" s="10" t="s">
         <v>374</v>
       </c>
-      <c r="D220" s="1" t="s">
-        <v>379</v>
-      </c>
-    </row>
-    <row r="221" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="B221" s="1" t="s">
+      <c r="D222" s="1" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="223" spans="1:21" ht="72" x14ac:dyDescent="0.3">
+      <c r="C223" s="49" t="s">
         <v>380</v>
-      </c>
-      <c r="C221" s="50" t="s">
-        <v>377</v>
-      </c>
-      <c r="D221" s="1" t="s">
-        <v>378</v>
-      </c>
-    </row>
-    <row r="222" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A222" s="10" t="s">
-        <v>375</v>
-      </c>
-      <c r="D222" s="1" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="223" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="C223" s="50" t="s">
-        <v>381</v>
       </c>
       <c r="D223" s="1" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="224" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A224" s="10" t="s">
+        <v>381</v>
+      </c>
+      <c r="D224" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="D224" s="1" t="s">
-        <v>383</v>
-      </c>
-    </row>
-    <row r="230" spans="1:21" x14ac:dyDescent="0.35">
+    </row>
+    <row r="230" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A230" s="3"/>
       <c r="B230" s="3"/>
       <c r="C230" s="4"/>
@@ -14218,31 +14213,31 @@
       <c r="S230" s="3"/>
       <c r="U230" s="3"/>
     </row>
-    <row r="231" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A231" s="1" t="s">
-        <v>357</v>
-      </c>
-      <c r="C231" s="46" t="s">
-        <v>355</v>
+        <v>356</v>
+      </c>
+      <c r="C231" s="45" t="s">
+        <v>354</v>
       </c>
       <c r="D231" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="232" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C232" s="50" t="s">
+        <v>385</v>
+      </c>
+      <c r="D232" s="1" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="232" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="C232" s="51" t="s">
-        <v>386</v>
-      </c>
-      <c r="D232" s="1" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="233" spans="1:21" ht="217.5" x14ac:dyDescent="0.35">
-      <c r="C233" s="51" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="235" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:21" ht="216" x14ac:dyDescent="0.3">
+      <c r="C233" s="50" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="235" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A235" s="3"/>
       <c r="B235" s="3"/>
       <c r="C235" s="4"/>
@@ -14261,77 +14256,77 @@
       <c r="S235" s="3"/>
       <c r="U235" s="3"/>
     </row>
-    <row r="236" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A236" s="1" t="s">
-        <v>358</v>
-      </c>
-      <c r="C236" s="46" t="s">
-        <v>353</v>
+        <v>357</v>
+      </c>
+      <c r="C236" s="45" t="s">
+        <v>352</v>
       </c>
       <c r="D236" s="1" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="237" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="237" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A237" s="10" t="s">
+        <v>389</v>
+      </c>
+      <c r="C237" s="50" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="238" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C238" s="50" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="239" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C239" s="50" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="240" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C240" s="50" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="241" spans="1:21" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C241" s="50" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="242" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C242" s="50" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="243" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A243" s="10" t="s">
         <v>390</v>
       </c>
-      <c r="C237" s="51" t="s">
-        <v>389</v>
-      </c>
-    </row>
-    <row r="238" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="C238" s="51" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="239" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="C239" s="51" t="s">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="240" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C240" s="51" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="241" spans="1:21" ht="32" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C241" s="51" t="s">
-        <v>403</v>
-      </c>
-    </row>
-    <row r="242" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="C242" s="51" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="243" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A243" s="10" t="s">
+      <c r="C243" s="50" t="s">
+        <v>392</v>
+      </c>
+      <c r="D243" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="C243" s="51" t="s">
+    </row>
+    <row r="244" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C244" s="50" t="s">
         <v>393</v>
       </c>
-      <c r="D243" s="1" t="s">
-        <v>392</v>
-      </c>
-    </row>
-    <row r="244" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="C244" s="51" t="s">
+    </row>
+    <row r="245" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C245" s="50" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="245" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="C245" s="51" t="s">
+    <row r="246" spans="1:21" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="C246" s="50" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="246" spans="1:21" ht="116" x14ac:dyDescent="0.35">
-      <c r="C246" s="51" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="249" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A249" s="3"/>
       <c r="B249" s="3"/>
       <c r="C249" s="4"/>
@@ -14350,34 +14345,34 @@
       <c r="S249" s="3"/>
       <c r="U249" s="3"/>
     </row>
-    <row r="250" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A250" s="1" t="s">
-        <v>367</v>
-      </c>
-      <c r="C250" s="46" t="s">
-        <v>354</v>
+        <v>366</v>
+      </c>
+      <c r="C250" s="45" t="s">
+        <v>353</v>
       </c>
       <c r="D250" s="1" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="251" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C251" s="50" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="251" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="C251" s="51" t="s">
+    <row r="252" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A252" s="10" t="s">
+        <v>399</v>
+      </c>
+      <c r="C252" s="50" t="s">
+        <v>400</v>
+      </c>
+      <c r="D252" s="1" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="252" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="A252" s="10" t="s">
-        <v>400</v>
-      </c>
-      <c r="C252" s="51" t="s">
-        <v>401</v>
-      </c>
-      <c r="D252" s="1" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="260" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A260" s="3"/>
       <c r="B260" s="3"/>
       <c r="C260" s="4"/>
@@ -14396,175 +14391,175 @@
       <c r="S260" s="3"/>
       <c r="U260" s="3"/>
     </row>
-    <row r="261" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A261" s="1" t="s">
-        <v>406</v>
-      </c>
-      <c r="C261" s="52" t="s">
+        <v>405</v>
+      </c>
+      <c r="C261" s="51" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="262" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A262" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="C262" s="50"/>
+      <c r="D262" s="1" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="263" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C263" s="50" t="s">
         <v>410</v>
       </c>
     </row>
-    <row r="262" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A262" s="10" t="s">
-        <v>408</v>
-      </c>
-      <c r="C262" s="51"/>
-      <c r="D262" s="1" t="s">
+    <row r="264" spans="1:21" ht="76.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B264" s="1" t="s">
+        <v>415</v>
+      </c>
+      <c r="C264" s="50" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="265" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C265" s="50" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="266" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C266" s="50" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="267" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C267" s="50" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="268" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A268" s="10" t="s">
         <v>409</v>
       </c>
-    </row>
-    <row r="263" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="C263" s="51" t="s">
-        <v>411</v>
-      </c>
-    </row>
-    <row r="264" spans="1:21" ht="76" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B264" s="1" t="s">
+      <c r="D268" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="C264" s="51" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="265" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="C265" s="51" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="266" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="C266" s="51" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="267" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="C267" s="51" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="268" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A268" s="10" t="s">
-        <v>410</v>
-      </c>
-      <c r="D268" s="1" t="s">
+    </row>
+    <row r="269" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="C269" s="50" t="s">
         <v>417</v>
       </c>
     </row>
-    <row r="269" spans="1:21" ht="58" x14ac:dyDescent="0.35">
-      <c r="C269" s="51" t="s">
+    <row r="270" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A270" s="35" t="s">
+        <v>419</v>
+      </c>
+      <c r="B270" s="36"/>
+      <c r="C270" s="52"/>
+      <c r="D270" s="38" t="s">
         <v>418</v>
       </c>
     </row>
-    <row r="270" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A270" s="35" t="s">
+    <row r="271" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A271" s="10" t="s">
         <v>420</v>
       </c>
-      <c r="B270" s="36"/>
-      <c r="C270" s="53"/>
-      <c r="D270" s="38" t="s">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="271" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A271" s="10" t="s">
+      <c r="D271" s="1" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="272" spans="1:21" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="C272" s="50" t="s">
         <v>421</v>
       </c>
-      <c r="D271" s="1" t="s">
+    </row>
+    <row r="273" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A273" s="10" t="s">
+        <v>425</v>
+      </c>
+      <c r="D273" s="1" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="272" spans="1:21" ht="130.5" x14ac:dyDescent="0.35">
-      <c r="C272" s="51" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="273" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A273" s="10" t="s">
+    <row r="274" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B274" s="50" t="s">
+        <v>424</v>
+      </c>
+      <c r="C274" s="50" t="s">
         <v>426</v>
       </c>
-      <c r="D273" s="1" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="274" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="B274" s="51" t="s">
-        <v>425</v>
-      </c>
-      <c r="C274" s="51" t="s">
+    </row>
+    <row r="275" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A275" s="10" t="s">
+        <v>428</v>
+      </c>
+      <c r="C275" s="50"/>
+      <c r="D275" s="1" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="275" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="A275" s="10" t="s">
+    <row r="276" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="C276" s="50" t="s">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="277" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A277" s="10" t="s">
         <v>429</v>
       </c>
-      <c r="C275" s="51"/>
-      <c r="D275" s="1" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="276" spans="1:21" ht="87" x14ac:dyDescent="0.35">
-      <c r="C276" s="51" t="s">
+      <c r="C277" s="50"/>
+      <c r="D277" s="1" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="278" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="C278" s="60" t="s">
         <v>432</v>
       </c>
     </row>
-    <row r="277" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="A277" s="10" t="s">
-        <v>430</v>
-      </c>
-      <c r="C277" s="51"/>
-      <c r="D277" s="1" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="278" spans="1:21" ht="87" x14ac:dyDescent="0.35">
-      <c r="C278" s="61" t="s">
+    <row r="279" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A279" s="19" t="s">
+        <v>434</v>
+      </c>
+      <c r="C279" s="20" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="280" spans="1:21" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="B280" s="50" t="s">
+        <v>435</v>
+      </c>
+      <c r="C280" s="50" t="s">
         <v>433</v>
       </c>
-    </row>
-    <row r="279" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A279" s="19" t="s">
-        <v>435</v>
-      </c>
-      <c r="C279" s="20" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="280" spans="1:21" ht="130.5" x14ac:dyDescent="0.35">
-      <c r="B280" s="51" t="s">
+      <c r="D280" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="C280" s="51" t="s">
-        <v>434</v>
-      </c>
-      <c r="D280" s="1" t="s">
+    </row>
+    <row r="281" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A281" s="10" t="s">
+        <v>438</v>
+      </c>
+      <c r="D281" s="1" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="282" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C282" s="50" t="s">
         <v>437</v>
       </c>
     </row>
-    <row r="281" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A281" s="10" t="s">
-        <v>439</v>
-      </c>
-      <c r="D281" s="1" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="282" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="C282" s="51" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="283" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A283" s="10" t="s">
-        <v>443</v>
-      </c>
-      <c r="C283" s="51"/>
-    </row>
-    <row r="284" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="C284" s="96" t="s">
         <v>442</v>
       </c>
-    </row>
-    <row r="287" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="C283" s="50"/>
+    </row>
+    <row r="284" spans="1:21" ht="72" x14ac:dyDescent="0.3">
+      <c r="C284" s="95" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="287" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A287" s="3"/>
       <c r="B287" s="3"/>
       <c r="C287" s="4"/>
@@ -14583,111 +14578,111 @@
       <c r="S287" s="3"/>
       <c r="U287" s="3"/>
     </row>
-    <row r="288" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="288" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A288" s="1" t="s">
-        <v>441</v>
-      </c>
-      <c r="C288" s="52" t="s">
+        <v>440</v>
+      </c>
+      <c r="C288" s="51" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="289" spans="1:21" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A289" s="55" t="s">
+        <v>503</v>
+      </c>
+      <c r="B289" s="59" t="s">
+        <v>507</v>
+      </c>
+      <c r="C289" s="57" t="s">
+        <v>506</v>
+      </c>
+      <c r="D289" s="58"/>
+    </row>
+    <row r="290" spans="1:21" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B290" s="53" t="s">
+        <v>482</v>
+      </c>
+      <c r="C290" s="50" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="289" spans="1:21" ht="73" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A289" s="56" t="s">
-        <v>504</v>
-      </c>
-      <c r="B289" s="60" t="s">
-        <v>508</v>
-      </c>
-      <c r="C289" s="58" t="s">
-        <v>507</v>
-      </c>
-      <c r="D289" s="59"/>
-    </row>
-    <row r="290" spans="1:21" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B290" s="54" t="s">
-        <v>483</v>
-      </c>
-      <c r="C290" s="51" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="291" spans="1:21" ht="58" x14ac:dyDescent="0.35">
-      <c r="A291" s="65" t="s">
+    <row r="291" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A291" s="64" t="s">
+        <v>538</v>
+      </c>
+      <c r="B291" s="65" t="s">
+        <v>537</v>
+      </c>
+      <c r="C291" s="66" t="s">
+        <v>447</v>
+      </c>
+      <c r="D291" s="67" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="292" spans="1:21" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A292" s="68"/>
+      <c r="B292" s="94" t="s">
+        <v>656</v>
+      </c>
+      <c r="C292" s="69"/>
+      <c r="D292" s="70"/>
+    </row>
+    <row r="293" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A293" s="64" t="s">
         <v>539</v>
       </c>
-      <c r="B291" s="66" t="s">
-        <v>538</v>
-      </c>
-      <c r="C291" s="67" t="s">
+      <c r="B293" s="65" t="s">
+        <v>536</v>
+      </c>
+      <c r="C293" s="66" t="s">
+        <v>446</v>
+      </c>
+      <c r="D293" s="67"/>
+    </row>
+    <row r="294" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A294" s="71"/>
+      <c r="B294" s="60" t="s">
         <v>448</v>
       </c>
-      <c r="D291" s="68" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="292" spans="1:21" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A292" s="69"/>
-      <c r="B292" s="95" t="s">
-        <v>657</v>
-      </c>
-      <c r="C292" s="70"/>
-      <c r="D292" s="71"/>
-    </row>
-    <row r="293" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="A293" s="65" t="s">
-        <v>540</v>
-      </c>
-      <c r="B293" s="66" t="s">
-        <v>537</v>
-      </c>
-      <c r="C293" s="67" t="s">
-        <v>447</v>
-      </c>
-      <c r="D293" s="68"/>
-    </row>
-    <row r="294" spans="1:21" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A294" s="72"/>
-      <c r="B294" s="61" t="s">
-        <v>449</v>
-      </c>
-      <c r="C294" s="54" t="s">
+      <c r="C294" s="53" t="s">
+        <v>498</v>
+      </c>
+      <c r="D294" s="72"/>
+    </row>
+    <row r="295" spans="1:21" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A295" s="73" t="s">
+        <v>443</v>
+      </c>
+      <c r="B295" s="74"/>
+      <c r="C295" s="75" t="s">
+        <v>445</v>
+      </c>
+      <c r="D295" s="70"/>
+    </row>
+    <row r="296" spans="1:21" ht="72" x14ac:dyDescent="0.3">
+      <c r="A296" s="19" t="s">
+        <v>463</v>
+      </c>
+      <c r="B296" s="53" t="s">
+        <v>501</v>
+      </c>
+      <c r="C296" s="20" t="s">
         <v>499</v>
       </c>
-      <c r="D294" s="73"/>
-    </row>
-    <row r="295" spans="1:21" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A295" s="74" t="s">
-        <v>444</v>
-      </c>
-      <c r="B295" s="75"/>
-      <c r="C295" s="76" t="s">
-        <v>446</v>
-      </c>
-      <c r="D295" s="71"/>
-    </row>
-    <row r="296" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A296" s="19" t="s">
-        <v>464</v>
-      </c>
-      <c r="B296" s="54" t="s">
-        <v>502</v>
-      </c>
-      <c r="C296" s="20" t="s">
+      <c r="D296" s="1" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="297" spans="1:21" ht="288" x14ac:dyDescent="0.3">
+      <c r="B297" s="1" t="s">
         <v>500</v>
       </c>
-      <c r="D296" s="1" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="297" spans="1:21" ht="290" x14ac:dyDescent="0.35">
-      <c r="B297" s="1" t="s">
-        <v>501</v>
-      </c>
-      <c r="C297" s="54" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="299" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="C297" s="53" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="299" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A299" s="3"/>
       <c r="B299" s="3"/>
       <c r="C299" s="4"/>
@@ -14706,63 +14701,63 @@
       <c r="S299" s="3"/>
       <c r="U299" s="3"/>
     </row>
-    <row r="300" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A300" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="C300" s="51"/>
+      <c r="D300" s="1" t="s">
         <v>452</v>
       </c>
-      <c r="C300" s="52"/>
-      <c r="D300" s="1" t="s">
+    </row>
+    <row r="301" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A301" s="10" t="s">
         <v>453</v>
       </c>
     </row>
-    <row r="301" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A301" s="10" t="s">
+    <row r="302" spans="1:21" ht="345.6" x14ac:dyDescent="0.3">
+      <c r="C302" s="53" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="303" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A303" s="19" t="s">
         <v>454</v>
       </c>
-    </row>
-    <row r="302" spans="1:21" ht="348" x14ac:dyDescent="0.35">
-      <c r="C302" s="54" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="303" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A303" s="19" t="s">
+      <c r="B303" s="41" t="s">
+        <v>459</v>
+      </c>
+      <c r="C303" s="50" t="s">
+        <v>462</v>
+      </c>
+      <c r="D303" s="1" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="304" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="C304" s="50" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="305" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A305" s="19" t="s">
         <v>455</v>
       </c>
-      <c r="B303" s="41" t="s">
+    </row>
+    <row r="306" spans="1:21" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="C306" s="50" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="307" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A307" s="19" t="s">
         <v>460</v>
       </c>
-      <c r="C303" s="51" t="s">
-        <v>463</v>
-      </c>
-      <c r="D303" s="1" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="304" spans="1:21" ht="58" x14ac:dyDescent="0.35">
-      <c r="C304" s="51" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="305" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A305" s="19" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="306" spans="1:21" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="C306" s="51" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="307" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A307" s="19" t="s">
+      <c r="C307" s="50" t="s">
         <v>461</v>
       </c>
-      <c r="C307" s="51" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="309" spans="1:21" x14ac:dyDescent="0.35">
+    </row>
+    <row r="309" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A309" s="3"/>
       <c r="B309" s="3"/>
       <c r="C309" s="4"/>
@@ -14781,81 +14776,81 @@
       <c r="S309" s="3"/>
       <c r="U309" s="3"/>
     </row>
-    <row r="310" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="310" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A310" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="C310" s="54" t="s">
+        <v>475</v>
+      </c>
+      <c r="D310" s="1" t="s">
         <v>465</v>
       </c>
-      <c r="C310" s="55" t="s">
+    </row>
+    <row r="311" spans="1:21" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A311" s="55" t="s">
+        <v>503</v>
+      </c>
+      <c r="B311" s="59" t="s">
+        <v>657</v>
+      </c>
+      <c r="C311" s="57" t="s">
+        <v>505</v>
+      </c>
+      <c r="D311" s="58"/>
+    </row>
+    <row r="312" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="C312" s="50" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="313" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A313" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="C313" s="60" t="s">
+        <v>540</v>
+      </c>
+      <c r="D313" s="1" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="314" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A314" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="C314" s="50"/>
+    </row>
+    <row r="315" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A315" s="1" t="s">
         <v>476</v>
       </c>
-      <c r="D310" s="1" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="311" spans="1:21" ht="58.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A311" s="56" t="s">
-        <v>504</v>
-      </c>
-      <c r="B311" s="60" t="s">
-        <v>658</v>
-      </c>
-      <c r="C311" s="58" t="s">
-        <v>506</v>
-      </c>
-      <c r="D311" s="59"/>
-    </row>
-    <row r="312" spans="1:21" ht="58" x14ac:dyDescent="0.35">
-      <c r="C312" s="51" t="s">
+      <c r="C315" s="50"/>
+    </row>
+    <row r="316" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A316" s="35" t="s">
+        <v>419</v>
+      </c>
+      <c r="B316" s="36"/>
+      <c r="C316" s="52"/>
+      <c r="D316" s="38" t="s">
         <v>467</v>
       </c>
     </row>
-    <row r="313" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A313" s="1" t="s">
-        <v>475</v>
-      </c>
-      <c r="C313" s="61" t="s">
-        <v>541</v>
-      </c>
-      <c r="D313" s="1" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="314" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A314" s="1" t="s">
-        <v>476</v>
-      </c>
-      <c r="C314" s="51"/>
-    </row>
-    <row r="315" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A315" s="1" t="s">
+    <row r="317" spans="1:21" ht="345.6" x14ac:dyDescent="0.3">
+      <c r="B317" s="53" t="s">
+        <v>479</v>
+      </c>
+      <c r="C317" s="95" t="s">
         <v>477</v>
       </c>
-      <c r="C315" s="51"/>
-    </row>
-    <row r="316" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A316" s="35" t="s">
-        <v>420</v>
-      </c>
-      <c r="B316" s="36"/>
-      <c r="C316" s="53"/>
-      <c r="D316" s="38" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="317" spans="1:21" ht="348" x14ac:dyDescent="0.35">
-      <c r="B317" s="54" t="s">
-        <v>480</v>
-      </c>
-      <c r="C317" s="96" t="s">
+    </row>
+    <row r="318" spans="1:21" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="C318" s="95" t="s">
         <v>478</v>
       </c>
     </row>
-    <row r="318" spans="1:21" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="C318" s="96" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="321" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="321" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A321" s="3"/>
       <c r="B321" s="3"/>
       <c r="C321" s="4"/>
@@ -14874,98 +14869,98 @@
       <c r="S321" s="3"/>
       <c r="U321" s="3"/>
     </row>
-    <row r="322" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="322" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A322" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="C322" s="54" t="s">
+        <v>484</v>
+      </c>
+      <c r="D322" s="1" t="s">
         <v>469</v>
       </c>
-      <c r="C322" s="55" t="s">
+    </row>
+    <row r="323" spans="1:21" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A323" s="55" t="s">
+        <v>503</v>
+      </c>
+      <c r="B323" s="56"/>
+      <c r="C323" s="57" t="s">
+        <v>504</v>
+      </c>
+      <c r="D323" s="58"/>
+    </row>
+    <row r="324" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B324" s="53" t="s">
+        <v>486</v>
+      </c>
+      <c r="C324" s="53" t="s">
+        <v>483</v>
+      </c>
+      <c r="D324" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="D322" s="1" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="323" spans="1:21" ht="29.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A323" s="56" t="s">
-        <v>504</v>
-      </c>
-      <c r="B323" s="57"/>
-      <c r="C323" s="58" t="s">
-        <v>505</v>
-      </c>
-      <c r="D323" s="59"/>
-    </row>
-    <row r="324" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="B324" s="54" t="s">
+    </row>
+    <row r="325" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A325" s="1" t="s">
+        <v>473</v>
+      </c>
+      <c r="B325" s="7" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="326" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A326" s="35" t="s">
+        <v>419</v>
+      </c>
+      <c r="B326" s="36"/>
+      <c r="C326" s="52"/>
+      <c r="D326" s="38" t="s">
         <v>487</v>
       </c>
-      <c r="C324" s="54" t="s">
-        <v>484</v>
-      </c>
-      <c r="D324" s="1" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="325" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="A325" s="1" t="s">
-        <v>474</v>
-      </c>
-      <c r="B325" s="7" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="326" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A326" s="35" t="s">
-        <v>420</v>
-      </c>
-      <c r="B326" s="36"/>
-      <c r="C326" s="53"/>
-      <c r="D326" s="38" t="s">
+    </row>
+    <row r="327" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A327" s="10" t="s">
         <v>488</v>
       </c>
     </row>
-    <row r="327" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A327" s="10" t="s">
+    <row r="328" spans="1:21" ht="144" x14ac:dyDescent="0.3">
+      <c r="C328" s="53" t="s">
         <v>489</v>
       </c>
     </row>
-    <row r="328" spans="1:21" ht="145" x14ac:dyDescent="0.35">
-      <c r="C328" s="54" t="s">
+    <row r="329" spans="1:21" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="C329" s="53" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="329" spans="1:21" ht="409.5" x14ac:dyDescent="0.35">
-      <c r="C329" s="54" t="s">
+    <row r="330" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A330" s="10" t="s">
         <v>491</v>
       </c>
-    </row>
-    <row r="330" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A330" s="10" t="s">
+      <c r="D330" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="D330" s="1" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="331" spans="1:21" ht="174" x14ac:dyDescent="0.35">
-      <c r="B331" s="54" t="s">
-        <v>498</v>
-      </c>
-      <c r="C331" s="54" t="s">
+    </row>
+    <row r="331" spans="1:21" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="B331" s="53" t="s">
         <v>497</v>
       </c>
-    </row>
-    <row r="332" spans="1:21" ht="348" x14ac:dyDescent="0.35">
-      <c r="C332" s="54" t="s">
+      <c r="C331" s="53" t="s">
         <v>496</v>
       </c>
     </row>
-    <row r="333" spans="1:21" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="C333" s="54" t="s">
+    <row r="332" spans="1:21" ht="345.6" x14ac:dyDescent="0.3">
+      <c r="C332" s="53" t="s">
         <v>495</v>
       </c>
     </row>
-    <row r="334" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="333" spans="1:21" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="C333" s="53" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="334" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A334" s="3"/>
       <c r="B334" s="3"/>
       <c r="C334" s="4"/>
@@ -14984,61 +14979,61 @@
       <c r="S334" s="3"/>
       <c r="U334" s="3"/>
     </row>
-    <row r="335" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="335" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A335" s="1" t="s">
+        <v>470</v>
+      </c>
+      <c r="C335" s="61" t="s">
+        <v>520</v>
+      </c>
+      <c r="D335" s="1" t="s">
         <v>471</v>
       </c>
-      <c r="C335" s="62" t="s">
-        <v>521</v>
-      </c>
-      <c r="D335" s="1" t="s">
+    </row>
+    <row r="336" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A336" s="10" t="s">
+        <v>509</v>
+      </c>
+      <c r="B336" s="7" t="s">
+        <v>512</v>
+      </c>
+      <c r="C336" s="53" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="337" spans="1:21" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="B337" s="60" t="s">
+        <v>518</v>
+      </c>
+      <c r="C337" s="50" t="s">
         <v>472</v>
       </c>
-    </row>
-    <row r="336" spans="1:21" ht="58" x14ac:dyDescent="0.35">
-      <c r="A336" s="10" t="s">
+      <c r="D337" s="1" t="s">
         <v>510</v>
       </c>
-      <c r="B336" s="7" t="s">
+    </row>
+    <row r="338" spans="1:21" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="B338" s="60" t="s">
+        <v>621</v>
+      </c>
+      <c r="C338" s="53" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="339" spans="1:21" ht="316.8" x14ac:dyDescent="0.3">
+      <c r="B339" s="60" t="s">
+        <v>620</v>
+      </c>
+      <c r="C339" s="60" t="s">
         <v>513</v>
       </c>
-      <c r="C336" s="54" t="s">
-        <v>512</v>
-      </c>
-    </row>
-    <row r="337" spans="1:21" ht="116" x14ac:dyDescent="0.35">
-      <c r="B337" s="61" t="s">
-        <v>519</v>
-      </c>
-      <c r="C337" s="51" t="s">
-        <v>473</v>
-      </c>
-      <c r="D337" s="1" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="338" spans="1:21" ht="174" x14ac:dyDescent="0.35">
-      <c r="B338" s="61" t="s">
-        <v>622</v>
-      </c>
-      <c r="C338" s="54" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="339" spans="1:21" ht="319" x14ac:dyDescent="0.35">
-      <c r="B339" s="61" t="s">
-        <v>621</v>
-      </c>
-      <c r="C339" s="61" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="340" spans="1:21" ht="174" x14ac:dyDescent="0.35">
-      <c r="C340" s="54" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="342" spans="1:21" x14ac:dyDescent="0.35">
+    </row>
+    <row r="340" spans="1:21" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="C340" s="53" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="342" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A342" s="3"/>
       <c r="B342" s="3"/>
       <c r="C342" s="4"/>
@@ -15057,28 +15052,28 @@
       <c r="S342" s="3"/>
       <c r="U342" s="3"/>
     </row>
-    <row r="343" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="343" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A343" s="1" t="s">
-        <v>471</v>
-      </c>
-      <c r="C343" s="62" t="s">
+        <v>470</v>
+      </c>
+      <c r="C343" s="61" t="s">
+        <v>514</v>
+      </c>
+      <c r="D343" s="1" t="s">
         <v>515</v>
       </c>
-      <c r="D343" s="1" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="344" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A344" s="63" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="345" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="C345" s="61" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="347" spans="1:21" x14ac:dyDescent="0.35">
+    </row>
+    <row r="344" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A344" s="62" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="345" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C345" s="60" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="347" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A347" s="3"/>
       <c r="B347" s="3"/>
       <c r="C347" s="4"/>
@@ -15097,105 +15092,105 @@
       <c r="S347" s="3"/>
       <c r="U347" s="3"/>
     </row>
-    <row r="348" spans="1:21" ht="29" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A348" s="1" t="s">
-        <v>517</v>
-      </c>
-      <c r="C348" s="62" t="s">
-        <v>520</v>
+        <v>516</v>
+      </c>
+      <c r="C348" s="61" t="s">
+        <v>519</v>
       </c>
       <c r="D348" s="1" t="s">
+        <v>569</v>
+      </c>
+    </row>
+    <row r="349" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A349" s="62" t="s">
+        <v>524</v>
+      </c>
+      <c r="B349" s="1" t="s">
         <v>570</v>
       </c>
-    </row>
-    <row r="349" spans="1:21" ht="87" x14ac:dyDescent="0.35">
-      <c r="A349" s="63" t="s">
+      <c r="C349" s="60" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="350" spans="1:21" ht="72" x14ac:dyDescent="0.3">
+      <c r="B350" s="60" t="s">
+        <v>522</v>
+      </c>
+      <c r="C350" s="60" t="s">
         <v>525</v>
       </c>
-      <c r="B349" s="1" t="s">
-        <v>571</v>
-      </c>
-      <c r="C349" s="61" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="350" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B350" s="61" t="s">
-        <v>523</v>
-      </c>
-      <c r="C350" s="61" t="s">
+    </row>
+    <row r="351" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A351" s="77" t="s">
+        <v>573</v>
+      </c>
+      <c r="B351" s="78"/>
+      <c r="C351" s="78"/>
+      <c r="D351" s="79"/>
+    </row>
+    <row r="352" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A352" s="80"/>
+      <c r="B352" s="60"/>
+      <c r="C352" s="60" t="s">
+        <v>574</v>
+      </c>
+      <c r="D352" s="81"/>
+    </row>
+    <row r="353" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A353" s="80"/>
+      <c r="B353" s="60"/>
+      <c r="C353" s="60" t="s">
+        <v>575</v>
+      </c>
+      <c r="D353" s="81"/>
+    </row>
+    <row r="354" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A354" s="80"/>
+      <c r="B354" s="60"/>
+      <c r="C354" s="60" t="s">
+        <v>576</v>
+      </c>
+      <c r="D354" s="81"/>
+    </row>
+    <row r="355" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A355" s="80"/>
+      <c r="B355" s="60"/>
+      <c r="C355" s="60" t="s">
+        <v>577</v>
+      </c>
+      <c r="D355" s="81"/>
+    </row>
+    <row r="356" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A356" s="82"/>
+      <c r="B356" s="83"/>
+      <c r="C356" s="83" t="s">
+        <v>578</v>
+      </c>
+      <c r="D356" s="84"/>
+    </row>
+    <row r="357" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A357" s="10" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="358" spans="1:21" ht="187.2" x14ac:dyDescent="0.3">
+      <c r="C358" s="60" t="s">
         <v>526</v>
       </c>
     </row>
-    <row r="351" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="A351" s="78" t="s">
-        <v>574</v>
-      </c>
-      <c r="B351" s="79"/>
-      <c r="C351" s="79"/>
-      <c r="D351" s="80"/>
-    </row>
-    <row r="352" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="A352" s="81"/>
-      <c r="B352" s="61"/>
-      <c r="C352" s="61" t="s">
-        <v>575</v>
-      </c>
-      <c r="D352" s="82"/>
-    </row>
-    <row r="353" spans="1:21" ht="58" x14ac:dyDescent="0.35">
-      <c r="A353" s="81"/>
-      <c r="B353" s="61"/>
-      <c r="C353" s="61" t="s">
-        <v>576</v>
-      </c>
-      <c r="D353" s="82"/>
-    </row>
-    <row r="354" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="A354" s="81"/>
-      <c r="B354" s="61"/>
-      <c r="C354" s="61" t="s">
-        <v>577</v>
-      </c>
-      <c r="D354" s="82"/>
-    </row>
-    <row r="355" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="A355" s="81"/>
-      <c r="B355" s="61"/>
-      <c r="C355" s="61" t="s">
-        <v>578</v>
-      </c>
-      <c r="D355" s="82"/>
-    </row>
-    <row r="356" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A356" s="83"/>
-      <c r="B356" s="84"/>
-      <c r="C356" s="84" t="s">
-        <v>579</v>
-      </c>
-      <c r="D356" s="85"/>
-    </row>
-    <row r="357" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A357" s="10" t="s">
-        <v>420</v>
-      </c>
-    </row>
-    <row r="358" spans="1:21" ht="188.5" x14ac:dyDescent="0.35">
-      <c r="C358" s="61" t="s">
+    <row r="359" spans="1:21" ht="316.8" x14ac:dyDescent="0.3">
+      <c r="C359" s="60" t="s">
         <v>527</v>
       </c>
     </row>
-    <row r="359" spans="1:21" ht="319" x14ac:dyDescent="0.35">
-      <c r="C359" s="61" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="360" spans="1:21" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="C360" s="61" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="362" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="360" spans="1:21" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="C360" s="60" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="362" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A362" s="3"/>
       <c r="B362" s="3"/>
       <c r="C362" s="4"/>
@@ -15214,82 +15209,82 @@
       <c r="S362" s="3"/>
       <c r="U362" s="3"/>
     </row>
-    <row r="363" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="363" spans="1:21" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A363" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="C363" s="61" t="s">
+        <v>543</v>
+      </c>
+      <c r="D363" s="1" t="s">
         <v>529</v>
       </c>
-      <c r="C363" s="62" t="s">
+    </row>
+    <row r="364" spans="1:21" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A364" s="55" t="s">
+        <v>503</v>
+      </c>
+      <c r="B364" s="56"/>
+      <c r="C364" s="63" t="s">
+        <v>535</v>
+      </c>
+      <c r="D364" s="58" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="365" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A365" s="10" t="s">
+        <v>530</v>
+      </c>
+      <c r="B365" s="1" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="366" spans="1:21" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="B366" s="60" t="s">
+        <v>622</v>
+      </c>
+      <c r="C366" s="60" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="367" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A367" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="D367" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="F367" s="10" t="s">
         <v>544</v>
       </c>
-      <c r="D363" s="1" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="364" spans="1:21" ht="73" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A364" s="56" t="s">
-        <v>504</v>
-      </c>
-      <c r="B364" s="57"/>
-      <c r="C364" s="64" t="s">
-        <v>536</v>
-      </c>
-      <c r="D364" s="59" t="s">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="365" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A365" s="10" t="s">
-        <v>531</v>
-      </c>
-      <c r="B365" s="1" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="366" spans="1:21" ht="87" x14ac:dyDescent="0.35">
-      <c r="B366" s="61" t="s">
-        <v>623</v>
-      </c>
-      <c r="C366" s="61" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="367" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A367" s="10" t="s">
-        <v>420</v>
-      </c>
-      <c r="D367" s="1" t="s">
-        <v>535</v>
-      </c>
-      <c r="F367" s="10" t="s">
+    </row>
+    <row r="368" spans="1:21" ht="172.8" x14ac:dyDescent="0.3">
+      <c r="C368" s="60" t="s">
+        <v>541</v>
+      </c>
+      <c r="H368" s="1" t="s">
         <v>545</v>
       </c>
     </row>
-    <row r="368" spans="1:21" ht="174" x14ac:dyDescent="0.35">
-      <c r="C368" s="61" t="s">
+    <row r="369" spans="1:21" ht="403.2" x14ac:dyDescent="0.3">
+      <c r="B369" s="90" t="s">
+        <v>639</v>
+      </c>
+      <c r="C369" s="60" t="s">
         <v>542</v>
       </c>
-      <c r="H368" s="1" t="s">
+      <c r="D369" s="1" t="s">
+        <v>548</v>
+      </c>
+      <c r="H369" s="1" t="s">
         <v>546</v>
       </c>
-    </row>
-    <row r="369" spans="1:21" ht="406" x14ac:dyDescent="0.35">
-      <c r="B369" s="91" t="s">
-        <v>640</v>
-      </c>
-      <c r="C369" s="61" t="s">
-        <v>543</v>
-      </c>
-      <c r="D369" s="1" t="s">
-        <v>549</v>
-      </c>
-      <c r="H369" s="1" t="s">
+      <c r="I369" s="1" t="s">
         <v>547</v>
       </c>
-      <c r="I369" s="1" t="s">
-        <v>548</v>
-      </c>
-    </row>
-    <row r="371" spans="1:21" x14ac:dyDescent="0.35">
+    </row>
+    <row r="371" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A371" s="3"/>
       <c r="B371" s="3"/>
       <c r="C371" s="4"/>
@@ -15308,26 +15303,26 @@
       <c r="S371" s="3"/>
       <c r="U371" s="3"/>
     </row>
-    <row r="372" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="372" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A372" s="1" t="s">
+        <v>549</v>
+      </c>
+      <c r="C372" s="61" t="s">
+        <v>551</v>
+      </c>
+      <c r="D372" s="1" t="s">
         <v>550</v>
       </c>
-      <c r="C372" s="62" t="s">
+    </row>
+    <row r="373" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A373" s="10" t="s">
+        <v>553</v>
+      </c>
+      <c r="C373" s="60" t="s">
         <v>552</v>
       </c>
-      <c r="D372" s="1" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="373" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="A373" s="10" t="s">
-        <v>554</v>
-      </c>
-      <c r="C373" s="61" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="375" spans="1:21" x14ac:dyDescent="0.35">
+    </row>
+    <row r="375" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A375" s="3"/>
       <c r="B375" s="3"/>
       <c r="C375" s="4"/>
@@ -15346,38 +15341,38 @@
       <c r="S375" s="3"/>
       <c r="U375" s="3"/>
     </row>
-    <row r="376" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="376" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A376" s="1" t="s">
+        <v>554</v>
+      </c>
+      <c r="C376" s="61" t="s">
+        <v>556</v>
+      </c>
+      <c r="D376" s="1" t="s">
         <v>555</v>
       </c>
-      <c r="C376" s="62" t="s">
+    </row>
+    <row r="377" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A377" s="10" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="378" spans="1:21" ht="72" x14ac:dyDescent="0.3">
+      <c r="C378" s="60" t="s">
         <v>557</v>
       </c>
-      <c r="D376" s="1" t="s">
-        <v>556</v>
-      </c>
-    </row>
-    <row r="377" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A377" s="10" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="378" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="C378" s="61" t="s">
+    </row>
+    <row r="379" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A379" s="10" t="s">
         <v>558</v>
       </c>
     </row>
-    <row r="379" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A379" s="10" t="s">
+    <row r="380" spans="1:21" ht="158.4" x14ac:dyDescent="0.3">
+      <c r="C380" s="60" t="s">
         <v>559</v>
       </c>
     </row>
-    <row r="380" spans="1:21" ht="159.5" x14ac:dyDescent="0.35">
-      <c r="C380" s="61" t="s">
-        <v>560</v>
-      </c>
-    </row>
-    <row r="382" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="382" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A382" s="3"/>
       <c r="B382" s="3"/>
       <c r="C382" s="4"/>
@@ -15396,52 +15391,52 @@
       <c r="S382" s="3"/>
       <c r="U382" s="3"/>
     </row>
-    <row r="383" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="383" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A383" s="1" t="s">
+        <v>560</v>
+      </c>
+      <c r="C383" s="61" t="s">
         <v>561</v>
       </c>
-      <c r="C383" s="62" t="s">
+      <c r="D383" s="1" t="s">
         <v>562</v>
       </c>
-      <c r="D383" s="1" t="s">
+    </row>
+    <row r="384" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="C384" s="60" t="s">
         <v>563</v>
       </c>
     </row>
-    <row r="384" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="C384" s="61" t="s">
+    <row r="385" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A385" s="10" t="s">
         <v>564</v>
       </c>
     </row>
-    <row r="385" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A385" s="10" t="s">
+    <row r="386" spans="1:21" ht="72" x14ac:dyDescent="0.3">
+      <c r="B386" s="60" t="s">
+        <v>567</v>
+      </c>
+      <c r="C386" s="60" t="s">
         <v>565</v>
       </c>
     </row>
-    <row r="386" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="B386" s="61" t="s">
+    <row r="387" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="B387" s="76" t="s">
         <v>568</v>
       </c>
-      <c r="C386" s="61" t="s">
+      <c r="C387" s="60" t="s">
         <v>566</v>
       </c>
     </row>
-    <row r="387" spans="1:21" ht="58" x14ac:dyDescent="0.35">
-      <c r="B387" s="77" t="s">
-        <v>569</v>
-      </c>
-      <c r="C387" s="61" t="s">
-        <v>567</v>
-      </c>
-    </row>
-    <row r="388" spans="1:21" ht="203" x14ac:dyDescent="0.35">
-      <c r="C388" s="91" t="s">
-        <v>639</v>
-      </c>
-      <c r="D388" s="91" t="s">
+    <row r="388" spans="1:21" ht="201.6" x14ac:dyDescent="0.3">
+      <c r="C388" s="90" t="s">
         <v>638</v>
       </c>
-    </row>
-    <row r="390" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="D388" s="90" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="390" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A390" s="3"/>
       <c r="B390" s="3"/>
       <c r="C390" s="4"/>
@@ -15460,53 +15455,53 @@
       <c r="S390" s="3"/>
       <c r="U390" s="3"/>
     </row>
-    <row r="391" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="391" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A391" s="1" t="s">
+        <v>571</v>
+      </c>
+      <c r="C391" s="61" t="s">
+        <v>581</v>
+      </c>
+      <c r="D391" s="1" t="s">
         <v>572</v>
       </c>
-      <c r="C391" s="62" t="s">
+    </row>
+    <row r="392" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C392" s="60" t="s">
+        <v>579</v>
+      </c>
+    </row>
+    <row r="393" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B393" s="60" t="s">
+        <v>583</v>
+      </c>
+      <c r="C393" s="60" t="s">
+        <v>580</v>
+      </c>
+    </row>
+    <row r="394" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A394" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="C394" s="60"/>
+    </row>
+    <row r="395" spans="1:21" ht="216" x14ac:dyDescent="0.3">
+      <c r="B395" s="91" t="s">
+        <v>642</v>
+      </c>
+      <c r="C395" s="90" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="396" spans="1:21" ht="273.60000000000002" x14ac:dyDescent="0.3">
+      <c r="C396" s="90" t="s">
+        <v>641</v>
+      </c>
+      <c r="D396" s="1" t="s">
         <v>582</v>
       </c>
-      <c r="D391" s="1" t="s">
-        <v>573</v>
-      </c>
-    </row>
-    <row r="392" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="C392" s="61" t="s">
-        <v>580</v>
-      </c>
-    </row>
-    <row r="393" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="B393" s="61" t="s">
-        <v>584</v>
-      </c>
-      <c r="C393" s="61" t="s">
-        <v>581</v>
-      </c>
-    </row>
-    <row r="394" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A394" s="10" t="s">
-        <v>420</v>
-      </c>
-      <c r="C394" s="61"/>
-    </row>
-    <row r="395" spans="1:21" ht="217.5" x14ac:dyDescent="0.35">
-      <c r="B395" s="92" t="s">
-        <v>643</v>
-      </c>
-      <c r="C395" s="91" t="s">
-        <v>641</v>
-      </c>
-    </row>
-    <row r="396" spans="1:21" ht="275.5" x14ac:dyDescent="0.35">
-      <c r="C396" s="91" t="s">
-        <v>642</v>
-      </c>
-      <c r="D396" s="1" t="s">
-        <v>583</v>
-      </c>
-    </row>
-    <row r="398" spans="1:21" x14ac:dyDescent="0.35">
+    </row>
+    <row r="398" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A398" s="3"/>
       <c r="B398" s="3"/>
       <c r="C398" s="4"/>
@@ -15525,80 +15520,80 @@
       <c r="S398" s="3"/>
       <c r="U398" s="3"/>
     </row>
-    <row r="399" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="399" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A399" s="1" t="s">
+        <v>584</v>
+      </c>
+      <c r="C399" s="61" t="s">
+        <v>586</v>
+      </c>
+      <c r="D399" s="1" t="s">
         <v>585</v>
       </c>
-      <c r="C399" s="62" t="s">
+    </row>
+    <row r="400" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A400" s="1" t="s">
+        <v>591</v>
+      </c>
+      <c r="B400" s="76" t="s">
+        <v>588</v>
+      </c>
+      <c r="C400" s="60" t="s">
         <v>587</v>
       </c>
-      <c r="D399" s="1" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="400" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A400" s="1" t="s">
+    </row>
+    <row r="401" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A401" s="1" t="s">
+        <v>590</v>
+      </c>
+      <c r="C401" s="60" t="s">
+        <v>593</v>
+      </c>
+      <c r="D401" s="1" t="s">
         <v>592</v>
       </c>
-      <c r="B400" s="77" t="s">
-        <v>589</v>
-      </c>
-      <c r="C400" s="61" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="401" spans="1:21" ht="58" x14ac:dyDescent="0.35">
-      <c r="A401" s="1" t="s">
-        <v>591</v>
-      </c>
-      <c r="C401" s="61" t="s">
+    </row>
+    <row r="402" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A402" s="1" t="s">
         <v>594</v>
       </c>
-      <c r="D401" s="1" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="402" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A402" s="1" t="s">
+      <c r="B402" s="1" t="s">
         <v>595</v>
       </c>
-      <c r="B402" s="1" t="s">
+      <c r="D402" s="1" t="s">
         <v>596</v>
       </c>
-      <c r="D402" s="1" t="s">
+    </row>
+    <row r="403" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A403" s="1" t="s">
         <v>597</v>
       </c>
-    </row>
-    <row r="403" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A403" s="1" t="s">
+      <c r="C403" s="60" t="s">
         <v>598</v>
       </c>
-      <c r="C403" s="61" t="s">
+    </row>
+    <row r="404" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A404" s="1" t="s">
+        <v>601</v>
+      </c>
+      <c r="C404" s="60" t="s">
+        <v>600</v>
+      </c>
+      <c r="D404" s="1" t="s">
         <v>599</v>
       </c>
     </row>
-    <row r="404" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="A404" s="1" t="s">
-        <v>602</v>
-      </c>
-      <c r="C404" s="61" t="s">
-        <v>601</v>
-      </c>
-      <c r="D404" s="1" t="s">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="405" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="405" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A405" s="10" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="406" spans="1:21" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="C406" s="60" t="s">
         <v>604</v>
       </c>
     </row>
-    <row r="406" spans="1:21" ht="116" x14ac:dyDescent="0.35">
-      <c r="C406" s="61" t="s">
-        <v>605</v>
-      </c>
-    </row>
-    <row r="408" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="408" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A408" s="3"/>
       <c r="B408" s="3"/>
       <c r="C408" s="4"/>
@@ -15617,175 +15612,175 @@
       <c r="S408" s="3"/>
       <c r="U408" s="3"/>
     </row>
-    <row r="409" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="409" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A409" s="1" t="s">
-        <v>590</v>
-      </c>
-      <c r="C409" s="62" t="s">
+        <v>589</v>
+      </c>
+      <c r="C409" s="61" t="s">
+        <v>616</v>
+      </c>
+      <c r="D409" s="1" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="410" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C410" s="60" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="411" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A411" s="77" t="s">
+        <v>419</v>
+      </c>
+      <c r="B411" s="85" t="s">
+        <v>619</v>
+      </c>
+      <c r="C411" s="78"/>
+      <c r="D411" s="79"/>
+    </row>
+    <row r="412" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A412" s="87" t="s">
+        <v>615</v>
+      </c>
+      <c r="C412" s="60"/>
+      <c r="D412" s="81"/>
+    </row>
+    <row r="413" spans="1:21" ht="316.8" x14ac:dyDescent="0.3">
+      <c r="A413" s="80"/>
+      <c r="B413" s="60" t="s">
+        <v>614</v>
+      </c>
+      <c r="C413" s="60" t="s">
+        <v>612</v>
+      </c>
+      <c r="D413" s="81" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="414" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A414" s="77" t="s">
         <v>617</v>
       </c>
-      <c r="D409" s="1" t="s">
-        <v>603</v>
-      </c>
-    </row>
-    <row r="410" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="C410" s="61" t="s">
+      <c r="B414" s="85"/>
+      <c r="C414" s="78"/>
+      <c r="D414" s="79"/>
+    </row>
+    <row r="415" spans="1:21" ht="374.4" x14ac:dyDescent="0.3">
+      <c r="A415" s="80"/>
+      <c r="C415" s="60" t="s">
+        <v>618</v>
+      </c>
+      <c r="D415" s="81"/>
+    </row>
+    <row r="416" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A416" s="77" t="s">
         <v>606</v>
       </c>
-    </row>
-    <row r="411" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A411" s="78" t="s">
-        <v>420</v>
-      </c>
-      <c r="B411" s="86" t="s">
-        <v>620</v>
-      </c>
-      <c r="C411" s="79"/>
-      <c r="D411" s="80"/>
-    </row>
-    <row r="412" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A412" s="88" t="s">
-        <v>616</v>
-      </c>
-      <c r="C412" s="61"/>
-      <c r="D412" s="82"/>
-    </row>
-    <row r="413" spans="1:21" ht="319" x14ac:dyDescent="0.35">
-      <c r="A413" s="81"/>
-      <c r="B413" s="61" t="s">
-        <v>615</v>
-      </c>
-      <c r="C413" s="61" t="s">
-        <v>613</v>
-      </c>
-      <c r="D413" s="82" t="s">
-        <v>614</v>
-      </c>
-    </row>
-    <row r="414" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A414" s="78" t="s">
-        <v>618</v>
-      </c>
-      <c r="B414" s="86"/>
-      <c r="C414" s="79"/>
-      <c r="D414" s="80"/>
-    </row>
-    <row r="415" spans="1:21" ht="377" x14ac:dyDescent="0.35">
-      <c r="A415" s="81"/>
-      <c r="C415" s="61" t="s">
-        <v>619</v>
-      </c>
-      <c r="D415" s="82"/>
-    </row>
-    <row r="416" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A416" s="78" t="s">
+      <c r="B416" s="85"/>
+      <c r="C416" s="86"/>
+      <c r="D416" s="79"/>
+    </row>
+    <row r="417" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A417" s="80"/>
+      <c r="C417" s="60" t="s">
         <v>607</v>
       </c>
-      <c r="B416" s="86"/>
-      <c r="C416" s="87"/>
-      <c r="D416" s="80"/>
-    </row>
-    <row r="417" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A417" s="81"/>
-      <c r="C417" s="61" t="s">
+      <c r="D417" s="81"/>
+    </row>
+    <row r="418" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A418" s="80"/>
+      <c r="C418" s="60" t="s">
         <v>608</v>
       </c>
-      <c r="D417" s="82"/>
-    </row>
-    <row r="418" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="A418" s="81"/>
-      <c r="C418" s="61" t="s">
+      <c r="D418" s="81"/>
+    </row>
+    <row r="419" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A419" s="80"/>
+      <c r="C419" s="60" t="s">
         <v>609</v>
       </c>
-      <c r="D418" s="82"/>
-    </row>
-    <row r="419" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A419" s="81"/>
-      <c r="C419" s="61" t="s">
+      <c r="D419" s="81"/>
+    </row>
+    <row r="420" spans="1:21" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A420" s="80"/>
+      <c r="C420" s="60" t="s">
         <v>610</v>
       </c>
-      <c r="D419" s="82"/>
-    </row>
-    <row r="420" spans="1:21" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A420" s="81"/>
-      <c r="C420" s="61" t="s">
+      <c r="D420" s="81"/>
+    </row>
+    <row r="421" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A421" s="87" t="s">
+        <v>419</v>
+      </c>
+      <c r="B421" s="1" t="s">
+        <v>625</v>
+      </c>
+      <c r="C421" s="60"/>
+      <c r="D421" s="81"/>
+    </row>
+    <row r="422" spans="1:21" ht="316.8" x14ac:dyDescent="0.3">
+      <c r="A422" s="82"/>
+      <c r="B422" s="88" t="s">
+        <v>624</v>
+      </c>
+      <c r="C422" s="83" t="s">
+        <v>623</v>
+      </c>
+      <c r="D422" s="84"/>
+    </row>
+    <row r="423" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A423" s="87" t="s">
+        <v>630</v>
+      </c>
+      <c r="B423" s="1" t="s">
+        <v>628</v>
+      </c>
+      <c r="C423" s="60"/>
+      <c r="D423" s="81"/>
+    </row>
+    <row r="424" spans="1:21" ht="388.8" x14ac:dyDescent="0.3">
+      <c r="A424" s="82"/>
+      <c r="B424" s="83" t="s">
+        <v>627</v>
+      </c>
+      <c r="C424" s="83" t="s">
+        <v>626</v>
+      </c>
+      <c r="D424" s="84"/>
+    </row>
+    <row r="425" spans="1:21" ht="72" x14ac:dyDescent="0.3">
+      <c r="A425" s="35" t="s">
+        <v>629</v>
+      </c>
+      <c r="B425" s="36"/>
+      <c r="C425" s="89" t="s">
         <v>611</v>
       </c>
-      <c r="D420" s="82"/>
-    </row>
-    <row r="421" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="A421" s="88" t="s">
-        <v>420</v>
-      </c>
-      <c r="B421" s="1" t="s">
-        <v>626</v>
-      </c>
-      <c r="C421" s="61"/>
-      <c r="D421" s="82"/>
-    </row>
-    <row r="422" spans="1:21" ht="319" x14ac:dyDescent="0.35">
-      <c r="A422" s="83"/>
-      <c r="B422" s="89" t="s">
-        <v>625</v>
-      </c>
-      <c r="C422" s="84" t="s">
-        <v>624</v>
-      </c>
-      <c r="D422" s="85"/>
-    </row>
-    <row r="423" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="A423" s="88" t="s">
+      <c r="D425" s="38"/>
+    </row>
+    <row r="426" spans="1:21" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A426" s="35" t="s">
         <v>631</v>
       </c>
-      <c r="B423" s="1" t="s">
-        <v>629</v>
-      </c>
-      <c r="C423" s="61"/>
-      <c r="D423" s="82"/>
-    </row>
-    <row r="424" spans="1:21" ht="391.5" x14ac:dyDescent="0.35">
-      <c r="A424" s="83"/>
-      <c r="B424" s="84" t="s">
-        <v>628</v>
-      </c>
-      <c r="C424" s="84" t="s">
-        <v>627</v>
-      </c>
-      <c r="D424" s="85"/>
-    </row>
-    <row r="425" spans="1:21" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A425" s="35" t="s">
-        <v>630</v>
-      </c>
-      <c r="B425" s="36"/>
-      <c r="C425" s="90" t="s">
-        <v>612</v>
-      </c>
-      <c r="D425" s="38"/>
-    </row>
-    <row r="426" spans="1:21" ht="58" x14ac:dyDescent="0.35">
-      <c r="A426" s="35" t="s">
+      <c r="B426" s="36"/>
+      <c r="C426" s="89" t="s">
         <v>632</v>
       </c>
-      <c r="B426" s="36"/>
-      <c r="C426" s="90" t="s">
+      <c r="D426" s="38"/>
+    </row>
+    <row r="427" spans="1:21" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A427" s="35" t="s">
         <v>633</v>
       </c>
-      <c r="D426" s="38"/>
-    </row>
-    <row r="427" spans="1:21" ht="29" x14ac:dyDescent="0.35">
-      <c r="A427" s="35" t="s">
+      <c r="B427" s="36" t="s">
+        <v>635</v>
+      </c>
+      <c r="C427" s="89" t="s">
         <v>634</v>
       </c>
-      <c r="B427" s="36" t="s">
-        <v>636</v>
-      </c>
-      <c r="C427" s="90" t="s">
-        <v>635</v>
-      </c>
       <c r="D427" s="38"/>
     </row>
-    <row r="430" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="430" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A430" s="3"/>
       <c r="B430" s="3"/>
       <c r="C430" s="4"/>
@@ -15804,101 +15799,101 @@
       <c r="S430" s="3"/>
       <c r="U430" s="3"/>
     </row>
-    <row r="431" spans="1:21" x14ac:dyDescent="0.35">
+    <row r="431" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A431" s="1" t="s">
-        <v>637</v>
-      </c>
-      <c r="C431" s="62"/>
-    </row>
-    <row r="432" spans="1:21" x14ac:dyDescent="0.35">
+        <v>636</v>
+      </c>
+      <c r="C431" s="61"/>
+    </row>
+    <row r="432" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A432" s="10" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="433" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A433" s="1" t="s">
         <v>644</v>
       </c>
-    </row>
-    <row r="433" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A433" s="1" t="s">
+      <c r="C433" s="92" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="434" spans="1:3" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A434" s="1" t="s">
         <v>645</v>
       </c>
-      <c r="C433" s="93" t="s">
+      <c r="C434" s="92" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="435" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A435" s="1" t="s">
+        <v>646</v>
+      </c>
+      <c r="C435" s="92" t="s">
         <v>648</v>
       </c>
     </row>
-    <row r="434" spans="1:3" ht="101.5" x14ac:dyDescent="0.35">
-      <c r="A434" s="1" t="s">
+    <row r="436" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A436" s="10" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="437" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A437" s="1" t="s">
+        <v>644</v>
+      </c>
+      <c r="C437" s="93" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="438" spans="1:3" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A438" s="1" t="s">
+        <v>645</v>
+      </c>
+      <c r="C438" s="93" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="439" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A439" s="1" t="s">
         <v>646</v>
       </c>
-      <c r="C434" s="93" t="s">
+      <c r="C439" s="92" t="s">
         <v>651</v>
       </c>
     </row>
-    <row r="435" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A435" s="1" t="s">
-        <v>647</v>
-      </c>
-      <c r="C435" s="93" t="s">
+    <row r="440" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A440" s="10" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="441" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A441" s="1" t="s">
+        <v>644</v>
+      </c>
+      <c r="C441" s="92" t="s">
         <v>649</v>
       </c>
     </row>
-    <row r="436" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A436" s="10" t="s">
-        <v>656</v>
-      </c>
-    </row>
-    <row r="437" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A437" s="1" t="s">
+    <row r="442" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="A442" s="1" t="s">
         <v>645</v>
       </c>
-      <c r="C437" s="94" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="438" spans="1:3" ht="58" x14ac:dyDescent="0.35">
-      <c r="A438" s="1" t="s">
+      <c r="C442" s="93" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="443" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A443" s="1" t="s">
         <v>646</v>
       </c>
-      <c r="C438" s="94" t="s">
-        <v>654</v>
-      </c>
-    </row>
-    <row r="439" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A439" s="1" t="s">
-        <v>647</v>
-      </c>
-      <c r="C439" s="93" t="s">
-        <v>652</v>
-      </c>
-    </row>
-    <row r="440" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A440" s="10" t="s">
-        <v>653</v>
-      </c>
-    </row>
-    <row r="441" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A441" s="1" t="s">
-        <v>645</v>
-      </c>
-      <c r="C441" s="93" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="442" spans="1:3" ht="87" x14ac:dyDescent="0.35">
-      <c r="A442" s="1" t="s">
-        <v>646</v>
-      </c>
-      <c r="C442" s="94" t="s">
-        <v>655</v>
-      </c>
-    </row>
-    <row r="443" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A443" s="1" t="s">
-        <v>647</v>
-      </c>
-      <c r="C443" s="93" t="s">
-        <v>652</v>
+      <c r="C443" s="92" t="s">
+        <v>651</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="26" type="noConversion"/>
+  <phoneticPr fontId="25" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="A101" r:id="rId1" xr:uid="{0889BDC3-4461-49B7-B3A7-5234BAE0C9D2}"/>
   </hyperlinks>

</xml_diff>